<commit_message>
used sum(), sumif() and sumifs()
</commit_message>
<xml_diff>
--- a/EXCEL/Cout Sum and Subtotal.xlsx
+++ b/EXCEL/Cout Sum and Subtotal.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/898af4500e89e0da/Desktop/DHRUV/Data Science and Analytics with GenAl/EXCEL/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="52" documentId="8_{32EB3D21-DB66-43B0-82E5-47AB2BC47EAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6FC31480-130F-41EE-8B71-23DA6A733934}"/>
+  <xr:revisionPtr revIDLastSave="76" documentId="8_{32EB3D21-DB66-43B0-82E5-47AB2BC47EAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1DA02301-1CEB-4C0F-902D-10FB83F7DA39}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" xr2:uid="{E39B28A0-9412-4544-BE2B-7A0C17A1740F}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="27">
   <si>
     <t>OrderID</t>
   </si>
@@ -108,13 +108,40 @@
   </si>
   <si>
     <t>countsifs (checks multiple conditions)</t>
+  </si>
+  <si>
+    <t>sumifs</t>
+  </si>
+  <si>
+    <t>sum(sum the whole selectes area</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">sumif   </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">  (sum according to one condition)</t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="16"/>
       <color theme="1"/>
@@ -126,6 +153,12 @@
       <b/>
       <sz val="16"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="16"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -151,7 +184,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -166,6 +199,9 @@
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -555,12 +591,12 @@
         <f>COUNT(D2:D11)</f>
         <v>9</v>
       </c>
-      <c r="K2" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="L2" s="5">
-        <f>COUNTIF(C2:C11,"North")</f>
-        <v>3</v>
+      <c r="K2" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="L2" s="6">
+        <f>SUM(D2:D11)</f>
+        <v>295300</v>
       </c>
     </row>
     <row r="3" spans="1:12" ht="126" x14ac:dyDescent="0.4">
@@ -589,12 +625,12 @@
         <f>COUNTA(C2:C11)</f>
         <v>10</v>
       </c>
-      <c r="K3" s="4" t="s">
-        <v>23</v>
+      <c r="K3" s="2" t="s">
+        <v>26</v>
       </c>
       <c r="L3">
-        <f>COUNTIFS(F2:F11,"Raj",C2:C11,"North",B2:B11,"Laptop")</f>
-        <v>1</v>
+        <f>SUMIF(C2:C11,"North",D2:D11)</f>
+        <v>65300</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.4">
@@ -623,8 +659,15 @@
         <f>COUNTBLANK(D2:E11)</f>
         <v>2</v>
       </c>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.4">
+      <c r="K4" t="s">
+        <v>24</v>
+      </c>
+      <c r="L4">
+        <f>SUMIFS(D2:D11,C2:C11,"North",B2:B11,"Laptop")</f>
+        <v>55000</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" ht="63" x14ac:dyDescent="0.4">
       <c r="A5" s="2">
         <v>1004</v>
       </c>
@@ -643,8 +686,15 @@
       <c r="F5" s="2" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.4">
+      <c r="H5" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="I5" s="5">
+        <f>COUNTIF(C2:C11,"North")</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" ht="84" x14ac:dyDescent="0.4">
       <c r="A6" s="2">
         <v>1005</v>
       </c>
@@ -662,6 +712,13 @@
       </c>
       <c r="F6" s="2" t="s">
         <v>11</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="I6">
+        <f>COUNTIFS(F2:F11,"Raj",C2:C11,"North",B2:B11,"Laptop")</f>
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.4">

</xml_diff>

<commit_message>
used subtotal() for dynamic sum
</commit_message>
<xml_diff>
--- a/EXCEL/Cout Sum and Subtotal.xlsx
+++ b/EXCEL/Cout Sum and Subtotal.xlsx
@@ -8,13 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/898af4500e89e0da/Desktop/DHRUV/Data Science and Analytics with GenAl/EXCEL/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="76" documentId="8_{32EB3D21-DB66-43B0-82E5-47AB2BC47EAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1DA02301-1CEB-4C0F-902D-10FB83F7DA39}"/>
+  <xr:revisionPtr revIDLastSave="126" documentId="8_{32EB3D21-DB66-43B0-82E5-47AB2BC47EAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B4C339D2-16F7-4527-96D9-059ACE928760}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" xr2:uid="{E39B28A0-9412-4544-BE2B-7A0C17A1740F}"/>
+    <workbookView minimized="1" xWindow="864" yWindow="696" windowWidth="17280" windowHeight="10500" xr2:uid="{E39B28A0-9412-4544-BE2B-7A0C17A1740F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$F$11</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -36,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="31">
   <si>
     <t>OrderID</t>
   </si>
@@ -108,9 +111,6 @@
   </si>
   <si>
     <t>countsifs (checks multiple conditions)</t>
-  </si>
-  <si>
-    <t>sumifs</t>
   </si>
   <si>
     <t>sum(sum the whole selectes area</t>
@@ -135,6 +135,21 @@
       </rPr>
       <t xml:space="preserve">  (sum according to one condition)</t>
     </r>
+  </si>
+  <si>
+    <t>sumifs  (according to multiple conditions)</t>
+  </si>
+  <si>
+    <t>Count</t>
+  </si>
+  <si>
+    <t>Sum</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Subtotal   </t>
+  </si>
+  <si>
+    <t>(it is a dynamic method to sum values)</t>
   </si>
 </sst>
 </file>
@@ -164,12 +179,30 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.749992370372631"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B0F0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -184,7 +217,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -195,13 +228,36 @@
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -538,14 +594,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4646335B-C91B-45B4-9F51-049F60B7F2E6}">
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:N11"/>
   <sheetFormatPr defaultRowHeight="21" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="8" max="8" width="9.92578125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="9.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -564,8 +620,19 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:12" ht="84" x14ac:dyDescent="0.4">
+      <c r="H1" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="13"/>
+      <c r="K1" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="L1" s="8"/>
+      <c r="N1" s="4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" ht="84" x14ac:dyDescent="0.4">
       <c r="A2" s="2">
         <v>1001</v>
       </c>
@@ -584,22 +651,26 @@
       <c r="F2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="H2" s="4" t="s">
+      <c r="H2" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="I2" s="5">
+      <c r="I2" s="15">
         <f>COUNT(D2:D11)</f>
         <v>9</v>
       </c>
-      <c r="K2" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="L2" s="6">
+      <c r="K2" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="L2" s="10">
         <f>SUM(D2:D11)</f>
         <v>295300</v>
       </c>
-    </row>
-    <row r="3" spans="1:12" ht="126" x14ac:dyDescent="0.4">
+      <c r="N2" s="5">
+        <f>SUBTOTAL(9,D2:D11)</f>
+        <v>295300</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" ht="126" x14ac:dyDescent="0.4">
       <c r="A3" s="2">
         <v>1002</v>
       </c>
@@ -618,22 +689,25 @@
       <c r="F3" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="H3" s="4" t="s">
+      <c r="H3" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="I3" s="5">
+      <c r="I3" s="15">
         <f>COUNTA(C2:C11)</f>
         <v>10</v>
       </c>
-      <c r="K3" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="L3">
+      <c r="K3" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="L3" s="11">
         <f>SUMIF(C2:C11,"North",D2:D11)</f>
         <v>65300</v>
       </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.4">
+      <c r="N3" s="6" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" ht="84" x14ac:dyDescent="0.4">
       <c r="A4" s="2">
         <v>1003</v>
       </c>
@@ -652,22 +726,22 @@
       <c r="F4" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="H4" t="s">
+      <c r="H4" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="I4" s="5">
+      <c r="I4" s="15">
         <f>COUNTBLANK(D2:E11)</f>
         <v>2</v>
       </c>
-      <c r="K4" t="s">
-        <v>24</v>
-      </c>
-      <c r="L4">
+      <c r="K4" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="L4" s="11">
         <f>SUMIFS(D2:D11,C2:C11,"North",B2:B11,"Laptop")</f>
         <v>55000</v>
       </c>
     </row>
-    <row r="5" spans="1:12" ht="63" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:14" ht="63" x14ac:dyDescent="0.4">
       <c r="A5" s="2">
         <v>1004</v>
       </c>
@@ -686,15 +760,15 @@
       <c r="F5" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="H5" s="4" t="s">
+      <c r="H5" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="I5" s="5">
+      <c r="I5" s="15">
         <f>COUNTIF(C2:C11,"North")</f>
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:12" ht="84" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:14" ht="84" x14ac:dyDescent="0.4">
       <c r="A6" s="2">
         <v>1005</v>
       </c>
@@ -713,15 +787,15 @@
       <c r="F6" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="H6" s="4" t="s">
+      <c r="H6" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="I6">
+      <c r="I6" s="15">
         <f>COUNTIFS(F2:F11,"Raj",C2:C11,"North",B2:B11,"Laptop")</f>
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A7" s="2">
         <v>1006</v>
       </c>
@@ -741,7 +815,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A8" s="2">
         <v>1007</v>
       </c>
@@ -761,7 +835,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A9" s="2">
         <v>1008</v>
       </c>
@@ -781,7 +855,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A10" s="2">
         <v>1009</v>
       </c>
@@ -801,7 +875,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A11" s="2">
         <v>1010</v>
       </c>

</xml_diff>